<commit_message>
Add six API cases for Week 4 automation practice
</commit_message>
<xml_diff>
--- a/repository-files/test-cases/test-cases.xlsx
+++ b/repository-files/test-cases/test-cases.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Case Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Steps" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tag Guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -357,7 +357,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="7">
     <tableColumn id="1" name="Case ID"/>
     <tableColumn id="2" name="Title"/>
@@ -372,7 +372,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" name="Case ID"/>
     <tableColumn id="2" name="Actions"/>
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="14" min="1" max="1"/>
@@ -1265,15 +1265,237 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="14"/>
-    <row r="21" ht="15" customHeight="1" s="14"/>
+    <row r="20" ht="210" customHeight="1" s="14">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>API-2009</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Completing a ride twice does not duplicate order history</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Verify that a second completion request for an already completed ride is rejected and leaves exactly one history entry for that ride, with the pre-existing history preserved. Use initialOrders and completedOrder to correlate history across requests. Check status, route, option ID and rejection against the stated requirements, not values derived from the response being checked.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>A fresh authorized sandbox session exists with all sandbox states disabled, no active ride and the three seeded history entries. Use the same bearer token and X-Sandbox-Session for all requests. Do not reset or replace the session between steps. The route is Oak Avenue to Market Street, using Yellow tariff ID 1. Run the existing per-test cleanup only after the final check; a reset between completion requests invalidates this scenario.</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>regression, api, negative, ride lifecycle</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>GET /orders
+POST /rides
+POST /rides/{rideId}/complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1" s="14">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>API-2010</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>An unknown ride option is rejected</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Verify that a ride request using an unknown ride option ID fails validation.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>A fresh authorized sandbox session exists with default settings and no active ride.</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>regression, api, negative</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>POST /rides</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1" s="14">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>API-2011</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>A seven-digit phone number is rejected</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Verify that requesting an OTP with fewer than eight phone digits fails validation.</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>The API is available. POST /auth/phone does not require a bearer token.</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>regression, api, negative</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>POST /auth/phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="72" customHeight="1" s="14">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>API-2012</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Malformed JSON in an OTP request is rejected</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Verify that the phone endpoint returns a defined error when the request body is invalid JSON.</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>The API is available. POST /auth/phone does not require a bearer token.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>regression, api, negative</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>POST /auth/phone</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1" s="14">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>API-2013</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Order history requires authorization</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Verify that an order-history request without an authorization token is rejected.</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>The API is available. Omit the Authorization header from the request.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>regression, api, negative</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>GET /orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="72" customHeight="1" s="14">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>API-2014</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Resolving the pickup location returns Oak Avenue</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Verify that the location endpoint returns the defined pickup address for an authorized request.</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>A fresh authorized sandbox session exists with default settings. Use its bearer token and X-Sandbox-Session.</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>regression, api</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>READY FOR AUTOMATION</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>POST /location/resolve</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G19">
+  <conditionalFormatting sqref="A2:G25">
     <cfRule type="expression" priority="1" dxfId="24">
       <formula>OR($F2="READY FOR AUTOMATION",$F2="BLOCKED",$F2="NEEDS_CLARIFICATION")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F19">
+  <conditionalFormatting sqref="F2:F25">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>OR($F2="READY FOR AUTOMATION",$F2="BLOCKED",$F2="NEEDS_CLARIFICATION")</formula>
     </cfRule>
@@ -1291,7 +1513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="14" min="1" max="1"/>
@@ -1676,12 +1898,120 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="14"/>
-    <row r="21" ht="15" customHeight="1" s="14"/>
+    <row r="20" ht="250" customHeight="1" s="14">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>API-2009</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>1. Send GET /orders. Retain the ordered collection as initialOrders.
+2. Send POST /rides with {"from":"Oak Avenue","to":"Market Street","rideOptionId":1}. Retain the returned ID as rideId.
+3. Send POST /rides/{rideId}/complete. Retain the returned order as completedOrder.
+4. Send POST /rides/{rideId}/complete again with the same captured ride ID.
+5. Send GET /orders using the same token and session.</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>1. HTTP 200 and exactly the three seeded orders defined by the supplied test data.
+2. HTTP 201, a positive ride ID, status driver_found, from Oak Avenue, to Market Street and option ID 1.
+3. HTTP 200. The returned ride has the captured rideId and status completed. The order has a positive ID absent from initialOrders, and its from/to values match the submitted route.
+4. HTTP 409 with error "Ride is missing or cannot be completed".
+5. HTTP 200 and exactly completedOrder followed by initialOrders: four entries, the new order once in first position, and every original entry preserved in its original relative order. The second completion creates no additional history entry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="72" customHeight="1" s="14">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>API-2010</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>1. Send POST /rides with the bearer token and body {"from":"Oak Avenue","to":"Market Street","rideOptionId":999}.</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>1. The response is HTTP 400 with error "Unknown ride option 999".</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1" s="14">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>API-2011</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>1. Send POST /auth/phone with Content-Type: application/json and body {"phone":"1234567"}.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>1. The response is HTTP 400 with error "Phone number must contain at least 8 digits".</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1" s="14">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>API-2012</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>1. Send POST /auth/phone with Content-Type: application/json and the raw body not-json (without surrounding quotes).</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>1. The response is HTTP 400 with error "Malformed request body".</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1" s="14">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>API-2013</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>1. Send GET /orders without an Authorization header.</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>1. The response is HTTP 401 with error "Missing or invalid token".</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1" s="14">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>API-2014</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>1. Send POST /location/resolve with the bearer token and no request body.</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>1. The response is HTTP 200 with location "Oak Avenue".</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:C19">
+  <conditionalFormatting sqref="A2:C25">
     <cfRule type="expression" priority="1" dxfId="24">
-      <formula>COUNTIFS('Case Summary'!$A$2:$A$19,$A2,'Case Summary'!$F$2:$F$19,"TODO")&gt;0</formula>
+      <formula>COUNTIFS('Case Summary'!$A$2:$A$25,$A2,'Case Summary'!$F$2:$F$25,"TODO")&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Keep only the two API cases needed for assignments
</commit_message>
<xml_diff>
--- a/repository-files/test-cases/test-cases.xlsx
+++ b/repository-files/test-cases/test-cases.xlsx
@@ -357,7 +357,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="7">
     <tableColumn id="1" name="Case ID"/>
     <tableColumn id="2" name="Title"/>
@@ -372,7 +372,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" name="Case ID"/>
     <tableColumn id="2" name="Actions"/>
@@ -579,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="14" min="1" max="1"/>
@@ -1341,161 +1341,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="72" customHeight="1" s="14">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>API-2011</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>A seven-digit phone number is rejected</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Verify that requesting an OTP with fewer than eight phone digits fails validation.</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>The API is available. POST /auth/phone does not require a bearer token.</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>regression, api, negative</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>READY FOR AUTOMATION</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>POST /auth/phone</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="72" customHeight="1" s="14">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>API-2012</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Malformed JSON in an OTP request is rejected</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Verify that the phone endpoint returns a defined error when the request body is invalid JSON.</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>The API is available. POST /auth/phone does not require a bearer token.</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>regression, api, negative</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>READY FOR AUTOMATION</t>
-        </is>
-      </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>POST /auth/phone</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="72" customHeight="1" s="14">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>API-2013</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Order history requires authorization</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Verify that an order-history request without an authorization token is rejected.</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>The API is available. Omit the Authorization header from the request.</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>regression, api, negative</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>READY FOR AUTOMATION</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>GET /orders</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="72" customHeight="1" s="14">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>API-2014</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Resolving the pickup location returns Oak Avenue</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Verify that the location endpoint returns the defined pickup address for an authorized request.</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>A fresh authorized sandbox session exists with default settings. Use its bearer token and X-Sandbox-Session.</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>regression, api</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>READY FOR AUTOMATION</t>
-        </is>
-      </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>POST /location/resolve</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:G25">
+  <conditionalFormatting sqref="A2:G21">
     <cfRule type="expression" priority="1" dxfId="24">
       <formula>OR($F2="READY FOR AUTOMATION",$F2="BLOCKED",$F2="NEEDS_CLARIFICATION")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F25">
+  <conditionalFormatting sqref="F2:F21">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>OR($F2="READY FOR AUTOMATION",$F2="BLOCKED",$F2="NEEDS_CLARIFICATION")</formula>
     </cfRule>
@@ -1513,7 +1365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="14" min="1" max="1"/>
@@ -1940,78 +1792,10 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1" s="14">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>API-2011</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>1. Send POST /auth/phone with Content-Type: application/json and body {"phone":"1234567"}.</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>1. The response is HTTP 400 with error "Phone number must contain at least 8 digits".</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1" s="14">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>API-2012</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>1. Send POST /auth/phone with Content-Type: application/json and the raw body not-json (without surrounding quotes).</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>1. The response is HTTP 400 with error "Malformed request body".</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1" s="14">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>API-2013</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>1. Send GET /orders without an Authorization header.</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>1. The response is HTTP 401 with error "Missing or invalid token".</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1" s="14">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>API-2014</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>1. Send POST /location/resolve with the bearer token and no request body.</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>1. The response is HTTP 200 with location "Oak Avenue".</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:C25">
+  <conditionalFormatting sqref="A2:C21">
     <cfRule type="expression" priority="1" dxfId="24">
-      <formula>COUNTIFS('Case Summary'!$A$2:$A$25,$A2,'Case Summary'!$F$2:$F$25,"TODO")&gt;0</formula>
+      <formula>COUNTIFS('Case Summary'!$A$2:$A$21,$A2,'Case Summary'!$F$2:$F$21,"TODO")&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Align Week 4 test case IDs with lesson order
</commit_message>
<xml_diff>
--- a/repository-files/test-cases/test-cases.xlsx
+++ b/repository-files/test-cases/test-cases.xlsx
@@ -1268,7 +1268,7 @@
     <row r="20" ht="210" customHeight="1" s="14">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>API-2009</t>
+          <t>API-2010</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="21" ht="72" customHeight="1" s="14">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>API-2010</t>
+          <t>API-2009</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1753,7 +1753,7 @@
     <row r="20" ht="250" customHeight="1" s="14">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>API-2009</t>
+          <t>API-2010</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1778,7 +1778,7 @@
     <row r="21" ht="72" customHeight="1" s="14">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>API-2010</t>
+          <t>API-2009</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">

</xml_diff>